<commit_message>
feat(ml): implement time-series demand forecasting with rule-based stock risk scoring
</commit_message>
<xml_diff>
--- a/backend/exports/orders.xlsx
+++ b/backend/exports/orders.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siparişler" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Siparişler" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Domates Salçası x2, Tarhana x1</t>
+          <t>Domates Salçası x2, Erişte x2, Gül suyu x1</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Organik Bal x1, Erişte x3</t>
+          <t>Organik Bal x1, Tarhana x2, Erişte x1</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,901 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Domates Salçası x1, Ev Yapımı Reçel x2, Erişte x1</t>
+          <t>Ev Yapımı Reçel x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Özlem Kılıç</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>250</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Domates Salçası x1, vişne reçeli x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Özlem Kılıç</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>120</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Domates Salçası x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Özlem Kılıç</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>260</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Organik Bal x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ayse Kaya</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>05320000001</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>640</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x2, Zeytinyağı  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mehmet Demir</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>05320000002</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>450</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Kestane Balı 450g x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fatma Celik</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>05320000003</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>780</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x3, Keçi Peyniri  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Özlem Kılıç</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>320</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Domates Salçası  x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fatih Yeğen</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>950</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x4, Kestane Balı 450g x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>İlkay</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>520</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x2, Bitki Çayı Papatya x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ahmet Kaya</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>5551000001</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>870</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x5, Biber Salçası 1kg x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ayşe Demir</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>5551000002</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>440</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Zeytinyağı  x1, Fındık  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mehmet Yılmaz</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5551000003</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>660</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ceviz İçi  x1, Tahin 800g x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fatma Çelik</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5551000004</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>720</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x6, Doğal Reçel Vişne x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ali Koç</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5551000005</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>820</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x3, Zeytin Siyah  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Zehra Arslan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>5551000006</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>540</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Kestane Balı 450g x1, Zeytin Yeşil  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Hüseyin Şahin</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5551000007</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>310</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x7, Pekmez 900g x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Elif Aydın</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5551000008</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>460</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Domates Salçası  x2, El Yapımı Mum x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Murat Öz</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>5551000009</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>980</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x4, Tulum Peyniri  x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Seda Akın</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5551000010</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>620</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x8, Kurutulmuş Domates x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Can Yıldız</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5551000011</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>540</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Kestane Balı 450g x2, Kurutulmuş Biber x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ece Tunç</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5551000012</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>430</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x9, Ayçiçek Yağı 5L x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Kerem Uçar</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5551000013</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>760</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x5, Ev Yapımı Erişte x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Nil Kara</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>5551000014</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>670</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Zeytinyağı  x2, Doğal Reçel Çilek x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Barış Eren</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5551000015</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>850</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x10, Nar Ekşisi 500ml x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gizem Kurt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5551000016</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>920</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Kestane Balı 450g x2, Bitki Çayı Adaçayı x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Tolga Deniz</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>5551000017</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>610</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x6, Doğal Sirke Elma x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Selin Güneş</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>5551000018</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>470</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x11, Kuru Kayısı 1kg x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Emre Acar</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5551000019</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>550</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Domates Salçası  x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Melis Ateş</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5551000020</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>720</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Keçi Peyniri  x7</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Burak Alp</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5551000021</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>810</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Türk Kahvesi x12</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Deniz Işık</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5551000022</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>390</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Tarhana 1kg x1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>İrem Bulut</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5551000023</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>640</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Zeytinyağı  x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Okan Efe</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5551000024</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>980</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Kestane Balı 450g x1, Türk Kahvesi x2</t>
         </is>
       </c>
     </row>

</xml_diff>